<commit_message>
Updated cosmetics and added a version number
</commit_message>
<xml_diff>
--- a/New_Relay_Onboarding_Form.xlsx
+++ b/New_Relay_Onboarding_Form.xlsx
@@ -3168,4 +3168,545 @@
   <pageSetup fitToHeight="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010076424A2F8899204F9FC29B11F01CF75E" ma:contentTypeVersion="46" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ef397cbb4cbecdae4f8d5c00b70fc449">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xmlns:ns3="78e23190-ffdc-4c9f-bb43-df7879b61858" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7eb136d3b0c600b3ab3eac7dab408951" ns1:_="" ns2:_="" ns3:_="">
+    <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
+    <xsd:import namespace="1570fe36-32a1-4b17-b77e-3b148eaac9e0"/>
+    <xsd:import namespace="78e23190-ffdc-4c9f-bb43-df7879b61858"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:Plant" minOccurs="0"/>
+                <xsd:element ref="ns2:System" minOccurs="0"/>
+                <xsd:element ref="ns2:FunctionalStructure" minOccurs="0"/>
+                <xsd:element ref="ns2:DocumentDescription"/>
+                <xsd:element ref="ns2:CreationDate" minOccurs="0"/>
+                <xsd:element ref="ns2:CurrentlyUesd" minOccurs="0"/>
+                <xsd:element ref="ns2:_Flow_SignoffStatus" minOccurs="0"/>
+                <xsd:element ref="ns2:Category" minOccurs="0"/>
+                <xsd:element ref="ns2:Reference" minOccurs="0"/>
+                <xsd:element ref="ns2:ReferenceNumber" minOccurs="0"/>
+                <xsd:element ref="ns2:d5b9f94c-ee4c-488b-8b26-8c1761682817State" minOccurs="0"/>
+                <xsd:element ref="ns2:d5b9f94c-ee4c-488b-8b26-8c1761682817City" minOccurs="0"/>
+                <xsd:element ref="ns2:d5b9f94c-ee4c-488b-8b26-8c1761682817PostalCode" minOccurs="0"/>
+                <xsd:element ref="ns2:d5b9f94c-ee4c-488b-8b26-8c1761682817Street" minOccurs="0"/>
+                <xsd:element ref="ns2:d5b9f94c-ee4c-488b-8b26-8c1761682817GeoLoc" minOccurs="0"/>
+                <xsd:element ref="ns2:d5b9f94c-ee4c-488b-8b26-8c1761682817DispName" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyProperties" minOccurs="0"/>
+                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyUIAction" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:d5b9f94c-ee4c-488b-8b26-8c1761682817CountryOrRegion" minOccurs="0"/>
+                <xsd:element ref="ns2:Categorypart2" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:CountryOrRegiond5b9f94c-ee4c-488b-8b26-8c1761682817" minOccurs="0"/>
+                <xsd:element ref="ns2:Stated5b9f94c-ee4c-488b-8b26-8c1761682817" minOccurs="0"/>
+                <xsd:element ref="ns2:Cityd5b9f94c-ee4c-488b-8b26-8c1761682817" minOccurs="0"/>
+                <xsd:element ref="ns2:PostalCoded5b9f94c-ee4c-488b-8b26-8c1761682817" minOccurs="0"/>
+                <xsd:element ref="ns2:Streetd5b9f94c-ee4c-488b-8b26-8c1761682817" minOccurs="0"/>
+                <xsd:element ref="ns2:GeoLocd5b9f94c-ee4c-488b-8b26-8c1761682817" minOccurs="0"/>
+                <xsd:element ref="ns2:DispNamed5b9f94c-ee4c-488b-8b26-8c1761682817" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="http://schemas.microsoft.com/sharepoint/v3" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="_ip_UnifiedCompliancePolicyProperties" ma:index="34" nillable="true" ma:displayName="Unified Compliance Policy Properties" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyProperties" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_ip_UnifiedCompliancePolicyUIAction" ma:index="35" nillable="true" ma:displayName="Unified Compliance Policy UI Action" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyUIAction" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="1570fe36-32a1-4b17-b77e-3b148eaac9e0" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="Plant" ma:index="2" nillable="true" ma:displayName="Plant" ma:description="The plant location " ma:internalName="Plant">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="System" ma:index="3" nillable="true" ma:displayName="System" ma:internalName="System" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="FunctionalStructure" ma:index="4" nillable="true" ma:displayName="Functional Structure " ma:format="Dropdown" ma:internalName="FunctionalStructure" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DocumentDescription" ma:index="5" ma:displayName="Document Description" ma:format="Dropdown" ma:internalName="DocumentDescription">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="CreationDate" ma:index="6" nillable="true" ma:displayName="Creation Date" ma:default="2020-03-08T00:00:00Z" ma:format="DateOnly" ma:internalName="CreationDate" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:DateTime"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="CurrentlyUesd" ma:index="7" nillable="true" ma:displayName="Active Document" ma:description="Is the fie a historical file kept for historical reasons, if it is applicable then select yes" ma:format="Dropdown" ma:internalName="CurrentlyUesd">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Choice">
+          <xsd:enumeration value="Yes"/>
+          <xsd:enumeration value="No"/>
+          <xsd:enumeration value="Latest"/>
+          <xsd:enumeration value="Superseded"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_Flow_SignoffStatus" ma:index="8" nillable="true" ma:displayName="Sign-off status" ma:internalName="Sign_x002d_off_x0020_status" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Category" ma:index="9" nillable="true" ma:displayName="Category" ma:format="Dropdown" ma:internalName="Category" ma:requiredMultiChoice="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoice">
+            <xsd:sequence>
+              <xsd:element name="Value" maxOccurs="unbounded" minOccurs="0" nillable="true">
+                <xsd:simpleType>
+                  <xsd:restriction base="dms:Choice">
+                    <xsd:enumeration value="Protection"/>
+                    <xsd:enumeration value="Project"/>
+                    <xsd:enumeration value="Maintenance"/>
+                    <xsd:enumeration value="Measurement"/>
+                    <xsd:enumeration value="Instrumentation"/>
+                    <xsd:enumeration value="Primary Plant"/>
+                    <xsd:enumeration value="none"/>
+                    <xsd:enumeration value="Electrical Protection"/>
+                    <xsd:enumeration value="Electronic Settings"/>
+                    <xsd:enumeration value="Manuals"/>
+                    <xsd:enumeration value="Work Guides"/>
+                    <xsd:enumeration value="Information"/>
+                    <xsd:enumeration value="Test Result"/>
+                    <xsd:enumeration value="Functional Description"/>
+                    <xsd:enumeration value="Drawing"/>
+                    <xsd:enumeration value="Report"/>
+                    <xsd:enumeration value="Circuit Breaker"/>
+                    <xsd:enumeration value="Generator"/>
+                    <xsd:enumeration value="Transformer"/>
+                    <xsd:enumeration value="Settings"/>
+                    <xsd:enumeration value="Electronic Test File"/>
+                    <xsd:enumeration value="License"/>
+                    <xsd:enumeration value="Calibration"/>
+                    <xsd:enumeration value="EIPC"/>
+                    <xsd:enumeration value="AVR"/>
+                    <xsd:enumeration value="Safety Critical Test"/>
+                    <xsd:enumeration value="Electronic Test File"/>
+                    <xsd:enumeration value="Standard"/>
+                    <xsd:enumeration value="Software"/>
+                  </xsd:restriction>
+                </xsd:simpleType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="Reference" ma:index="10" nillable="true" ma:displayName="Reference" ma:description="A reference to the document in SAP or DMS" ma:format="Dropdown" ma:internalName="Reference">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Choice">
+          <xsd:enumeration value="DMS"/>
+          <xsd:enumeration value="WO number"/>
+          <xsd:enumeration value="SAP - M3"/>
+          <xsd:enumeration value="Notification"/>
+          <xsd:enumeration value="Meridian"/>
+          <xsd:enumeration value="Functional Location"/>
+          <xsd:enumeration value="PMPR"/>
+          <xsd:enumeration value="Calibration"/>
+          <xsd:enumeration value="MOC"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="ReferenceNumber" ma:index="11" nillable="true" ma:displayName="Reference Number" ma:format="Dropdown" ma:internalName="ReferenceNumber" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="d5b9f94c-ee4c-488b-8b26-8c1761682817State" ma:index="12" nillable="true" ma:displayName="Plant: State" ma:hidden="true" ma:internalName="State" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="d5b9f94c-ee4c-488b-8b26-8c1761682817City" ma:index="13" nillable="true" ma:displayName="Plant: City" ma:hidden="true" ma:internalName="City" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="d5b9f94c-ee4c-488b-8b26-8c1761682817PostalCode" ma:index="14" nillable="true" ma:displayName="Plant: Postal Code" ma:hidden="true" ma:internalName="PostalCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="d5b9f94c-ee4c-488b-8b26-8c1761682817Street" ma:index="15" nillable="true" ma:displayName="Plant: Street" ma:hidden="true" ma:internalName="Street" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="d5b9f94c-ee4c-488b-8b26-8c1761682817GeoLoc" ma:index="16" nillable="true" ma:displayName="Plant: Coordinates" ma:hidden="true" ma:internalName="GeoLoc" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="d5b9f94c-ee4c-488b-8b26-8c1761682817DispName" ma:index="17" nillable="true" ma:displayName="Name" ma:description="" ma:hidden="true" ma:internalName="DispName" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="20" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="21" nillable="true" ma:displayName="Tags" ma:hidden="true" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="22" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="23" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="24" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="25" nillable="true" ma:displayName="KeyPoints" ma:hidden="true" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="26" nillable="true" ma:displayName="Extracted Text" ma:hidden="true" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="30" nillable="true" ma:displayName="Location" ma:hidden="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="33" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="36" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="d5b9f94c-ee4c-488b-8b26-8c1761682817CountryOrRegion" ma:index="38" nillable="true" ma:displayName="Plant: Country/Region" ma:hidden="true" ma:internalName="CountryOrRegion" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Categorypart2" ma:index="39" nillable="true" ma:displayName="Category part 2" ma:description="An additional Category Tag to further define your data" ma:format="Dropdown" ma:hidden="true" ma:internalName="Categorypart2" ma:readOnly="false">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Choice">
+          <xsd:enumeration value="Primary Plant"/>
+          <xsd:enumeration value="Protection"/>
+          <xsd:enumeration value="Settings"/>
+          <xsd:enumeration value="400V"/>
+          <xsd:enumeration value="6.6kV"/>
+          <xsd:enumeration value="11kV"/>
+          <xsd:enumeration value="Transformer"/>
+          <xsd:enumeration value="Circuit breaker"/>
+          <xsd:enumeration value="Choice 9"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="41" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="94d5a718-e02a-4652-97a0-3645cb65c432" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="43" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="44" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="45" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="CountryOrRegiond5b9f94c-ee4c-488b-8b26-8c1761682817" ma:index="46" nillable="true" ma:displayName="Plant: Country/Region" ma:internalName="CountryOrRegion0" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Stated5b9f94c-ee4c-488b-8b26-8c1761682817" ma:index="47" nillable="true" ma:displayName="Plant: State" ma:internalName="State0" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Cityd5b9f94c-ee4c-488b-8b26-8c1761682817" ma:index="48" nillable="true" ma:displayName="Plant: City" ma:internalName="City0" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="PostalCoded5b9f94c-ee4c-488b-8b26-8c1761682817" ma:index="49" nillable="true" ma:displayName="Plant: Postal Code" ma:internalName="PostalCode0" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Streetd5b9f94c-ee4c-488b-8b26-8c1761682817" ma:index="50" nillable="true" ma:displayName="Plant: Street" ma:internalName="Street0" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="GeoLocd5b9f94c-ee4c-488b-8b26-8c1761682817" ma:index="51" nillable="true" ma:displayName="Plant: Coordinates" ma:internalName="GeoLoc0" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DispNamed5b9f94c-ee4c-488b-8b26-8c1761682817" ma:index="52" nillable="true" ma:displayName="Plant: Name" ma:internalName="DispName0" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="78e23190-ffdc-4c9f-bb43-df7879b61858" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="27" nillable="true" ma:displayName="Shared With" ma:hidden="true" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="28" nillable="true" ma:displayName="Shared With Details" ma:hidden="true" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="42" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c20b481c-2a83-4c3d-8e12-daa4dd5859a1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="78e23190-ffdc-4c9f-bb43-df7879b61858">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="1" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="78e23190-ffdc-4c9f-bb43-df7879b61858" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Categorypart2 xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <System xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0">Protection Relay</System>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <DocumentDescription xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0">Check sheets for Protection relays </DocumentDescription>
+    <Category xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0"/>
+    <Reference xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <FunctionalStructure xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <ReferenceNumber xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <Plant xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0">{"DisplayName":"Geothermal","EntityType":"Custom"}</Plant>
+    <CreationDate xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0">2026-06-03T07:00:00+00:00</CreationDate>
+    <CurrentlyUesd xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0">Latest</CurrentlyUesd>
+    <d5b9f94c-ee4c-488b-8b26-8c1761682817PostalCode xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <d5b9f94c-ee4c-488b-8b26-8c1761682817DispName xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0">Geothermal</d5b9f94c-ee4c-488b-8b26-8c1761682817DispName>
+    <d5b9f94c-ee4c-488b-8b26-8c1761682817CountryOrRegion xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <d5b9f94c-ee4c-488b-8b26-8c1761682817State xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <d5b9f94c-ee4c-488b-8b26-8c1761682817City xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <d5b9f94c-ee4c-488b-8b26-8c1761682817Street xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+    <d5b9f94c-ee4c-488b-8b26-8c1761682817GeoLoc xmlns="1570fe36-32a1-4b17-b77e-3b148eaac9e0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D0E1039-FE98-4FF2-ADD2-00F4B2769C2C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5B262E4-385D-4B49-8A3C-970214C80B65}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DAE7094-359E-488B-B272-0ACD4FDFF748}"/>
 </file>
</xml_diff>